<commit_message>
Update DTR RODGE.xlsx and related documentation with new SHA-256 hashes. Modify audit templates and runtime manifests to reflect changes in source and runtime files. Adjust AuriMark component to include logo image and update style snapshots in DTR CSC form manifest.
</commit_message>
<xml_diff>
--- a/templates/runtime/dtr-csc-form-48-v1.xlsx
+++ b/templates/runtime/dtr-csc-form-48-v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\DTR - PDS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SystemFiles\CursorProjects\Auri\templates\source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C92AFB35-AF5C-4DE0-ABF4-21D5195E2B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5193266A-70C8-45E0-B4F2-6AA674B3F347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="6660" yWindow="885" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>DPSU</author>
   </authors>
   <commentList>
-    <comment ref="P12" authorId="0" shapeId="0">
+    <comment ref="P12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -417,25 +417,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -451,7 +442,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -487,37 +477,15 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -534,6 +502,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -546,8 +541,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,11 +577,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1008,7 +1003,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1024,1135 +1019,1135 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="67" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
     </row>
     <row r="2" spans="1:16" ht="3.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="43"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="19"/>
-      <c r="B3" s="68" t="s">
+      <c r="A3" s="15"/>
+      <c r="B3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="68" t="s">
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="21"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="63"/>
+      <c r="M3" s="63"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="17"/>
     </row>
     <row r="4" spans="1:16" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="15"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="13"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="11"/>
     </row>
     <row r="5" spans="1:16" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
     </row>
     <row r="6" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65"/>
-      <c r="B6" s="65"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="65" t="str">
+      <c r="A6" s="60"/>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="60" t="str">
         <f>A6</f>
       </c>
-      <c r="J6" s="65"/>
-      <c r="K6" s="65"/>
-      <c r="L6" s="65"/>
-      <c r="M6" s="65"/>
-      <c r="N6" s="65"/>
-      <c r="O6" s="65"/>
+      <c r="J6" s="60"/>
+      <c r="K6" s="60"/>
+      <c r="L6" s="60"/>
+      <c r="M6" s="60"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="60"/>
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="66" t="s">
+      <c r="A7" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="66"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="66"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="66" t="s">
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="66"/>
-      <c r="K7" s="66"/>
-      <c r="L7" s="66"/>
-      <c r="M7" s="66"/>
-      <c r="N7" s="66"/>
-      <c r="O7" s="66"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="61"/>
+      <c r="L7" s="61"/>
+      <c r="M7" s="61"/>
+      <c r="N7" s="61"/>
+      <c r="O7" s="61"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="44" t="s">
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="45"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="48" t="str">
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="43" t="str">
         <f>D8</f>
       </c>
-      <c r="M8" s="48"/>
-      <c r="N8" s="48"/>
-      <c r="O8" s="48"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="18" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="46"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="22" t="s">
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="18" t="s">
         <v>15</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="N9" s="46"/>
-      <c r="O9" s="46"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="16" t="s">
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="23" t="s">
+      <c r="E10" s="12"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="16" t="s">
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="M10" s="16"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="46"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="32"/>
+      <c r="O10" s="32"/>
     </row>
     <row r="11" spans="1:16" ht="4.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="23"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="50" t="s">
+      <c r="A12" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="62"/>
-      <c r="D12" s="61" t="s">
+      <c r="C12" s="58"/>
+      <c r="D12" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="62"/>
-      <c r="F12" s="58" t="s">
+      <c r="E12" s="58"/>
+      <c r="F12" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="59"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="63" t="s">
+      <c r="G12" s="55"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="J12" s="60" t="s">
+      <c r="J12" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="K12" s="58"/>
-      <c r="L12" s="61" t="s">
+      <c r="K12" s="54"/>
+      <c r="L12" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="M12" s="62"/>
-      <c r="N12" s="58" t="s">
+      <c r="M12" s="58"/>
+      <c r="N12" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="O12" s="59"/>
+      <c r="O12" s="55"/>
       <c r="P12" s="3"/>
     </row>
     <row r="13" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="51"/>
-      <c r="B13" s="32" t="s">
+      <c r="A13" s="46"/>
+      <c r="B13" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="29" t="s">
+      <c r="F13" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="25" t="s">
+      <c r="H13" s="7"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="K13" s="26" t="s">
+      <c r="K13" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="L13" s="32" t="s">
+      <c r="L13" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M13" s="33" t="s">
+      <c r="M13" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="N13" s="29" t="s">
+      <c r="N13" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="O13" s="25" t="s">
+      <c r="O13" s="21" t="s">
         <v>8</v>
       </c>
       <c r="P13" s="3"/>
     </row>
     <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="24">
+      <c r="A14" s="20">
         <v>1</v>
       </c>
       <c r="B14" s="34"/>
       <c r="C14" s="35"/>
       <c r="D14" s="34"/>
       <c r="E14" s="35"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="24">
+      <c r="F14" s="36"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="20">
         <v>1</v>
       </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="7"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="40"/>
       <c r="L14" s="34"/>
       <c r="M14" s="35"/>
-      <c r="N14" s="30"/>
-      <c r="O14" s="6"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="37"/>
       <c r="P14" s="3"/>
     </row>
     <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="24">
+      <c r="A15" s="20">
         <v>2</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="24">
+      <c r="B15" s="38"/>
+      <c r="C15" s="39"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="20">
         <v>2</v>
       </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="30"/>
-      <c r="O15" s="6"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="42"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="39"/>
+      <c r="N15" s="36"/>
+      <c r="O15" s="37"/>
       <c r="P15" s="3"/>
     </row>
     <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="24">
+      <c r="A16" s="20">
         <v>3</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="24">
+      <c r="B16" s="38"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="20">
         <v>3</v>
       </c>
-      <c r="J16" s="4"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="36"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="6"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="42"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="36"/>
+      <c r="O16" s="37"/>
       <c r="P16" s="3"/>
     </row>
     <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="24">
+      <c r="A17" s="20">
         <v>4</v>
       </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="24">
+      <c r="B17" s="38"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="20">
         <v>4</v>
       </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="27"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="30"/>
-      <c r="O17" s="6"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="39"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="37"/>
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="24">
+      <c r="A18" s="20">
         <v>5</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="24">
+      <c r="B18" s="38"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="20">
         <v>5</v>
       </c>
-      <c r="J18" s="4"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="6"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="36"/>
+      <c r="O18" s="37"/>
       <c r="P18" s="3"/>
     </row>
     <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="24">
+      <c r="A19" s="20">
         <v>6</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="24">
+      <c r="B19" s="38"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="20">
         <v>6</v>
       </c>
-      <c r="J19" s="4"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="37"/>
-      <c r="N19" s="30"/>
-      <c r="O19" s="6"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="42"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="36"/>
+      <c r="O19" s="37"/>
       <c r="P19" s="3"/>
     </row>
     <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="24">
+      <c r="A20" s="20">
         <v>7</v>
       </c>
       <c r="B20" s="34"/>
       <c r="C20" s="35"/>
       <c r="D20" s="34"/>
       <c r="E20" s="35"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="24">
+      <c r="F20" s="36"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="20">
         <v>7</v>
       </c>
-      <c r="J20" s="6"/>
-      <c r="K20" s="7"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="40"/>
       <c r="L20" s="34"/>
       <c r="M20" s="35"/>
-      <c r="N20" s="30"/>
-      <c r="O20" s="6"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="37"/>
       <c r="P20" s="3"/>
     </row>
     <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="24">
+      <c r="A21" s="20">
         <v>8</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="24">
+      <c r="B21" s="38"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="20">
         <v>8</v>
       </c>
-      <c r="J21" s="4"/>
-      <c r="K21" s="7"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="40"/>
       <c r="L21" s="34"/>
       <c r="M21" s="35"/>
-      <c r="N21" s="30"/>
-      <c r="O21" s="6"/>
+      <c r="N21" s="36"/>
+      <c r="O21" s="37"/>
       <c r="P21" s="3"/>
     </row>
     <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="24">
+      <c r="A22" s="20">
         <v>9</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="24">
+      <c r="B22" s="38"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="20">
         <v>9</v>
       </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="37"/>
-      <c r="N22" s="30"/>
-      <c r="O22" s="6"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="42"/>
+      <c r="L22" s="38"/>
+      <c r="M22" s="39"/>
+      <c r="N22" s="36"/>
+      <c r="O22" s="37"/>
       <c r="P22" s="3"/>
     </row>
     <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="24">
+      <c r="A23" s="20">
         <v>10</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="24">
+      <c r="B23" s="38"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="20">
         <v>10</v>
       </c>
-      <c r="J23" s="4"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="37"/>
-      <c r="N23" s="30"/>
-      <c r="O23" s="6"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="42"/>
+      <c r="L23" s="38"/>
+      <c r="M23" s="39"/>
+      <c r="N23" s="36"/>
+      <c r="O23" s="37"/>
       <c r="P23" s="3"/>
     </row>
     <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="24">
+      <c r="A24" s="20">
         <v>11</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="24">
+      <c r="B24" s="38"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="20">
         <v>11</v>
       </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="27"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="6"/>
+      <c r="J24" s="41"/>
+      <c r="K24" s="42"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="39"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="37"/>
       <c r="P24" s="3"/>
     </row>
     <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="24">
+      <c r="A25" s="20">
         <v>12</v>
       </c>
-      <c r="B25" s="38"/>
-      <c r="C25" s="39"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="24">
+      <c r="B25" s="34"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="20">
         <v>12</v>
       </c>
-      <c r="J25" s="13"/>
-      <c r="K25" s="28"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="39"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="13"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="40"/>
+      <c r="L25" s="34"/>
+      <c r="M25" s="35"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="37"/>
       <c r="P25" s="3"/>
     </row>
     <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="24">
+      <c r="A26" s="20">
         <v>13</v>
       </c>
       <c r="B26" s="34"/>
       <c r="C26" s="35"/>
       <c r="D26" s="34"/>
       <c r="E26" s="35"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="24">
+      <c r="F26" s="36"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="20">
         <v>13</v>
       </c>
-      <c r="J26" s="6"/>
-      <c r="K26" s="7"/>
+      <c r="J26" s="37"/>
+      <c r="K26" s="40"/>
       <c r="L26" s="34"/>
       <c r="M26" s="35"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="6"/>
+      <c r="N26" s="36"/>
+      <c r="O26" s="37"/>
       <c r="P26" s="3"/>
     </row>
     <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="24">
+      <c r="A27" s="20">
         <v>14</v>
       </c>
       <c r="B27" s="34"/>
       <c r="C27" s="35"/>
       <c r="D27" s="34"/>
       <c r="E27" s="35"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="24">
+      <c r="F27" s="36"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="20">
         <v>14</v>
       </c>
-      <c r="J27" s="6"/>
-      <c r="K27" s="7"/>
+      <c r="J27" s="37"/>
+      <c r="K27" s="40"/>
       <c r="L27" s="34"/>
       <c r="M27" s="35"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="6"/>
+      <c r="N27" s="36"/>
+      <c r="O27" s="37"/>
       <c r="P27" s="3"/>
     </row>
     <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="24">
+      <c r="A28" s="20">
         <v>15</v>
       </c>
-      <c r="B28" s="36"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="37"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="24">
+      <c r="B28" s="38"/>
+      <c r="C28" s="39"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="20">
         <v>15</v>
       </c>
-      <c r="J28" s="4"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="36"/>
-      <c r="M28" s="37"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="6"/>
+      <c r="J28" s="41"/>
+      <c r="K28" s="42"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="39"/>
+      <c r="N28" s="36"/>
+      <c r="O28" s="37"/>
       <c r="P28" s="3"/>
     </row>
     <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="24">
+      <c r="A29" s="20">
         <v>16</v>
       </c>
-      <c r="B29" s="36"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="37"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="24">
+      <c r="B29" s="38"/>
+      <c r="C29" s="39"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="20">
         <v>16</v>
       </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="36"/>
-      <c r="M29" s="37"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="6"/>
+      <c r="J29" s="41"/>
+      <c r="K29" s="42"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="39"/>
+      <c r="N29" s="36"/>
+      <c r="O29" s="37"/>
       <c r="P29" s="3"/>
     </row>
     <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="24">
+      <c r="A30" s="20">
         <v>17</v>
       </c>
-      <c r="B30" s="36"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="37"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="24">
+      <c r="B30" s="38"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="37"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="20">
         <v>17</v>
       </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="36"/>
-      <c r="M30" s="37"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="6"/>
+      <c r="J30" s="41"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="39"/>
+      <c r="N30" s="36"/>
+      <c r="O30" s="37"/>
       <c r="P30" s="3"/>
     </row>
     <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="24">
+      <c r="A31" s="20">
         <v>18</v>
       </c>
-      <c r="B31" s="36"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="24">
+      <c r="B31" s="38"/>
+      <c r="C31" s="39"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="37"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="20">
         <v>18</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="36"/>
-      <c r="M31" s="37"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="6"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="42"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="39"/>
+      <c r="N31" s="36"/>
+      <c r="O31" s="37"/>
       <c r="P31" s="3"/>
     </row>
     <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="24">
+      <c r="A32" s="20">
         <v>19</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="37"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="24">
+      <c r="B32" s="38"/>
+      <c r="C32" s="39"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="37"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="20">
         <v>19</v>
       </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="36"/>
-      <c r="M32" s="37"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="6"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="42"/>
+      <c r="L32" s="38"/>
+      <c r="M32" s="39"/>
+      <c r="N32" s="36"/>
+      <c r="O32" s="37"/>
       <c r="P32" s="3"/>
     </row>
     <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="24">
+      <c r="A33" s="20">
         <v>20</v>
       </c>
       <c r="B33" s="34"/>
       <c r="C33" s="35"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="24">
+      <c r="D33" s="38"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="20">
         <v>20</v>
       </c>
-      <c r="J33" s="6"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="36"/>
-      <c r="M33" s="37"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="6"/>
+      <c r="J33" s="37"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="39"/>
+      <c r="N33" s="36"/>
+      <c r="O33" s="37"/>
       <c r="P33" s="3"/>
     </row>
     <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="24">
+      <c r="A34" s="20">
         <v>21</v>
       </c>
       <c r="B34" s="34"/>
       <c r="C34" s="35"/>
       <c r="D34" s="34"/>
       <c r="E34" s="35"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="24">
+      <c r="F34" s="36"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="20">
         <v>21</v>
       </c>
-      <c r="J34" s="6"/>
-      <c r="K34" s="7"/>
+      <c r="J34" s="37"/>
+      <c r="K34" s="40"/>
       <c r="L34" s="34"/>
       <c r="M34" s="35"/>
-      <c r="N34" s="30"/>
-      <c r="O34" s="6"/>
+      <c r="N34" s="36"/>
+      <c r="O34" s="37"/>
       <c r="P34" s="3"/>
     </row>
     <row r="35" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="24">
+      <c r="A35" s="20">
         <v>22</v>
       </c>
-      <c r="B35" s="36"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="24">
+      <c r="B35" s="38"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="20">
         <v>22</v>
       </c>
-      <c r="J35" s="4"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="36"/>
-      <c r="M35" s="37"/>
-      <c r="N35" s="30"/>
-      <c r="O35" s="6"/>
+      <c r="J35" s="41"/>
+      <c r="K35" s="42"/>
+      <c r="L35" s="38"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="36"/>
+      <c r="O35" s="37"/>
       <c r="P35" s="3"/>
     </row>
     <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="24">
+      <c r="A36" s="20">
         <v>23</v>
       </c>
-      <c r="B36" s="36"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="37"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="24">
+      <c r="B36" s="38"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="37"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="20">
         <v>23</v>
       </c>
-      <c r="J36" s="4"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="36"/>
-      <c r="M36" s="37"/>
-      <c r="N36" s="30"/>
-      <c r="O36" s="6"/>
+      <c r="J36" s="41"/>
+      <c r="K36" s="42"/>
+      <c r="L36" s="38"/>
+      <c r="M36" s="39"/>
+      <c r="N36" s="36"/>
+      <c r="O36" s="37"/>
       <c r="P36" s="3"/>
     </row>
     <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="24">
+      <c r="A37" s="20">
         <v>24</v>
       </c>
-      <c r="B37" s="36"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="24">
+      <c r="B37" s="38"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="37"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="20">
         <v>24</v>
       </c>
-      <c r="J37" s="4"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="36"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="30"/>
-      <c r="O37" s="6"/>
+      <c r="J37" s="41"/>
+      <c r="K37" s="42"/>
+      <c r="L37" s="38"/>
+      <c r="M37" s="39"/>
+      <c r="N37" s="36"/>
+      <c r="O37" s="37"/>
       <c r="P37" s="3"/>
     </row>
     <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="24">
+      <c r="A38" s="20">
         <v>25</v>
       </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="37"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="24">
+      <c r="B38" s="38"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="37"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="20">
         <v>25</v>
       </c>
-      <c r="J38" s="4"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="36"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="30"/>
-      <c r="O38" s="6"/>
+      <c r="J38" s="41"/>
+      <c r="K38" s="42"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="36"/>
+      <c r="O38" s="37"/>
       <c r="P38" s="3"/>
     </row>
     <row r="39" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="24">
+      <c r="A39" s="20">
         <v>26</v>
       </c>
-      <c r="B39" s="36"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="30"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="24">
+      <c r="B39" s="38"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="39"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="37"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="20">
         <v>26</v>
       </c>
-      <c r="J39" s="4"/>
-      <c r="K39" s="27"/>
-      <c r="L39" s="36"/>
-      <c r="M39" s="37"/>
-      <c r="N39" s="30"/>
-      <c r="O39" s="6"/>
+      <c r="J39" s="41"/>
+      <c r="K39" s="42"/>
+      <c r="L39" s="38"/>
+      <c r="M39" s="39"/>
+      <c r="N39" s="36"/>
+      <c r="O39" s="37"/>
       <c r="P39" s="3"/>
     </row>
     <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="24">
+      <c r="A40" s="20">
         <v>27</v>
       </c>
-      <c r="B40" s="36"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="24">
+      <c r="B40" s="38"/>
+      <c r="C40" s="39"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="39"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="20">
         <v>27</v>
       </c>
-      <c r="J40" s="4"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="36"/>
-      <c r="M40" s="37"/>
-      <c r="N40" s="30"/>
-      <c r="O40" s="6"/>
+      <c r="J40" s="41"/>
+      <c r="K40" s="42"/>
+      <c r="L40" s="38"/>
+      <c r="M40" s="39"/>
+      <c r="N40" s="36"/>
+      <c r="O40" s="37"/>
       <c r="P40" s="3"/>
     </row>
     <row r="41" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="24">
+      <c r="A41" s="20">
         <v>28</v>
       </c>
       <c r="B41" s="34"/>
       <c r="C41" s="35"/>
       <c r="D41" s="34"/>
       <c r="E41" s="35"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="24">
+      <c r="F41" s="36"/>
+      <c r="G41" s="37"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="20">
         <v>28</v>
       </c>
-      <c r="J41" s="6"/>
-      <c r="K41" s="7"/>
+      <c r="J41" s="37"/>
+      <c r="K41" s="40"/>
       <c r="L41" s="34"/>
       <c r="M41" s="35"/>
-      <c r="N41" s="30"/>
-      <c r="O41" s="6"/>
+      <c r="N41" s="36"/>
+      <c r="O41" s="37"/>
       <c r="P41" s="3"/>
     </row>
     <row r="42" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="24">
+      <c r="A42" s="20">
         <v>29</v>
       </c>
-      <c r="B42" s="36"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="36"/>
-      <c r="E42" s="37"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="24">
+      <c r="B42" s="38"/>
+      <c r="C42" s="39"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="37"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="20">
         <v>29</v>
       </c>
-      <c r="J42" s="4"/>
-      <c r="K42" s="27"/>
-      <c r="L42" s="36"/>
-      <c r="M42" s="37"/>
-      <c r="N42" s="30"/>
-      <c r="O42" s="6"/>
+      <c r="J42" s="41"/>
+      <c r="K42" s="42"/>
+      <c r="L42" s="38"/>
+      <c r="M42" s="39"/>
+      <c r="N42" s="36"/>
+      <c r="O42" s="37"/>
       <c r="P42" s="3"/>
     </row>
     <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="24">
+      <c r="A43" s="20">
         <v>30</v>
       </c>
       <c r="B43" s="34"/>
       <c r="C43" s="35"/>
       <c r="D43" s="34"/>
       <c r="E43" s="35"/>
-      <c r="F43" s="30"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="24">
+      <c r="F43" s="36"/>
+      <c r="G43" s="37"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="20">
         <v>30</v>
       </c>
-      <c r="J43" s="6"/>
-      <c r="K43" s="7"/>
+      <c r="J43" s="37"/>
+      <c r="K43" s="40"/>
       <c r="L43" s="34"/>
       <c r="M43" s="35"/>
-      <c r="N43" s="30"/>
-      <c r="O43" s="6"/>
+      <c r="N43" s="36"/>
+      <c r="O43" s="37"/>
       <c r="P43" s="3"/>
     </row>
     <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="24">
+      <c r="A44" s="20">
         <v>31</v>
       </c>
       <c r="B44" s="34"/>
       <c r="C44" s="35"/>
       <c r="D44" s="34"/>
       <c r="E44" s="35"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="24">
+      <c r="F44" s="36"/>
+      <c r="G44" s="37"/>
+      <c r="H44" s="8"/>
+      <c r="I44" s="20">
         <v>31</v>
       </c>
-      <c r="J44" s="6"/>
-      <c r="K44" s="7"/>
+      <c r="J44" s="37"/>
+      <c r="K44" s="40"/>
       <c r="L44" s="34"/>
       <c r="M44" s="35"/>
-      <c r="N44" s="30"/>
-      <c r="O44" s="6"/>
+      <c r="N44" s="36"/>
+      <c r="O44" s="37"/>
       <c r="P44" s="3"/>
     </row>
     <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="54" t="s">
+      <c r="A45" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="B45" s="55"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="57"/>
-      <c r="F45" s="47">
+      <c r="B45" s="51"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="52"/>
+      <c r="E45" s="53"/>
+      <c r="F45" s="33">
         <f>SUM(F14:F44)</f>
         <v>0</v>
       </c>
-      <c r="G45" s="40"/>
-      <c r="H45" s="42"/>
-      <c r="I45" s="54" t="s">
+      <c r="G45" s="26"/>
+      <c r="H45" s="28"/>
+      <c r="I45" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="J45" s="56"/>
-      <c r="K45" s="56"/>
-      <c r="L45" s="56"/>
-      <c r="M45" s="57"/>
-      <c r="N45" s="47">
+      <c r="J45" s="52"/>
+      <c r="K45" s="52"/>
+      <c r="L45" s="52"/>
+      <c r="M45" s="53"/>
+      <c r="N45" s="33">
         <f>SUM(N14:N44)</f>
         <v>0</v>
       </c>
-      <c r="O45" s="40"/>
+      <c r="O45" s="26"/>
       <c r="P45" s="3"/>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="H46" s="12"/>
+      <c r="H46" s="9"/>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="H47" s="12"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="H48" s="12"/>
+      <c r="H48" s="9"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H49" s="12"/>
+      <c r="H49" s="9"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H50" s="12"/>
+      <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H51" s="12"/>
+      <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H52" s="12"/>
+      <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:15" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="49" t="str">
+      <c r="A53" s="44" t="str">
         <f>A6</f>
       </c>
-      <c r="B53" s="49"/>
-      <c r="C53" s="49"/>
-      <c r="D53" s="49"/>
-      <c r="E53" s="49"/>
-      <c r="F53" s="49"/>
-      <c r="G53" s="49"/>
-      <c r="H53" s="12"/>
-      <c r="I53" s="49" t="str">
+      <c r="B53" s="44"/>
+      <c r="C53" s="44"/>
+      <c r="D53" s="44"/>
+      <c r="E53" s="44"/>
+      <c r="F53" s="44"/>
+      <c r="G53" s="44"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="44" t="str">
         <f>A6</f>
       </c>
-      <c r="J53" s="49"/>
-      <c r="K53" s="49"/>
-      <c r="L53" s="49"/>
-      <c r="M53" s="49"/>
-      <c r="N53" s="49"/>
-      <c r="O53" s="49"/>
+      <c r="J53" s="44"/>
+      <c r="K53" s="44"/>
+      <c r="L53" s="44"/>
+      <c r="M53" s="44"/>
+      <c r="N53" s="44"/>
+      <c r="O53" s="44"/>
     </row>
     <row r="54" spans="1:15" ht="3.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="12"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="12"/>
-      <c r="I54" s="12"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
-      <c r="L54" s="12"/>
-      <c r="M54" s="12"/>
-      <c r="N54" s="12"/>
-      <c r="O54" s="12"/>
+      <c r="A54" s="9"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="9"/>
+      <c r="J54" s="9"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="9"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9"/>
+      <c r="O54" s="9"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A55" s="12"/>
-      <c r="B55" s="12" t="s">
+      <c r="A55" s="9"/>
+      <c r="B55" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="12" t="s">
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="27"/>
+      <c r="I55" s="9"/>
+      <c r="J55" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="K55" s="12"/>
-      <c r="L55" s="12"/>
-      <c r="M55" s="12"/>
-      <c r="N55" s="12"/>
-      <c r="O55" s="12"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="9"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="9"/>
+      <c r="O55" s="9"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A56" s="12"/>
-      <c r="B56" s="12"/>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="12"/>
-      <c r="F56" s="12"/>
-      <c r="G56" s="12"/>
-      <c r="H56" s="12"/>
-      <c r="I56" s="12"/>
-      <c r="J56" s="12"/>
-      <c r="K56" s="12"/>
-      <c r="L56" s="12"/>
-      <c r="M56" s="12"/>
-      <c r="N56" s="12"/>
-      <c r="O56" s="12"/>
+      <c r="A56" s="9"/>
+      <c r="B56" s="9"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="9"/>
+      <c r="J56" s="9"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="9"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9"/>
+      <c r="O56" s="9"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="H57" s="12"/>
+      <c r="H57" s="9"/>
     </row>
     <row r="58" spans="1:15" ht="12" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="5"/>
-      <c r="B58" s="5"/>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
-      <c r="H58" s="12"/>
-      <c r="I58" s="5"/>
-      <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
-      <c r="L58" s="5"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="5"/>
-      <c r="O58" s="5"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="9"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
     </row>
     <row r="59" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="52" t="s">
+      <c r="B59" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="14"/>
-      <c r="J59" s="52" t="s">
+      <c r="C59" s="59"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="59"/>
+      <c r="F59" s="59"/>
+      <c r="G59" s="6"/>
+      <c r="H59" s="10"/>
+      <c r="J59" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="K59" s="52"/>
-      <c r="L59" s="52"/>
-      <c r="M59" s="52"/>
-      <c r="N59" s="52"/>
-      <c r="O59" s="9"/>
+      <c r="K59" s="59"/>
+      <c r="L59" s="59"/>
+      <c r="M59" s="59"/>
+      <c r="N59" s="59"/>
+      <c r="O59" s="6"/>
     </row>
     <row r="60" spans="1:15" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F60" s="53"/>
-      <c r="G60" s="53"/>
-      <c r="H60" s="8"/>
-      <c r="N60" s="53"/>
-      <c r="O60" s="53"/>
+      <c r="F60" s="49"/>
+      <c r="G60" s="49"/>
+      <c r="H60" s="5"/>
+      <c r="N60" s="49"/>
+      <c r="O60" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -2174,13 +2169,13 @@
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="J59:N59"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="L8:O8"/>
     <mergeCell ref="A53:G53"/>
     <mergeCell ref="I53:O53"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="J59:N59"/>
     <mergeCell ref="I12:I13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2194,7 +2189,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
@@ -2205,7 +2200,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>

</xml_diff>